<commit_message>
Added test results for the integration between movement and vision modules
</commit_message>
<xml_diff>
--- a/test/AssignmentAndWorkOrder_test.xlsx
+++ b/test/AssignmentAndWorkOrder_test.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{F124E770-FCEE-C145-BB87-981F54A33F30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{336CA497-929E-8E43-ACC0-3AB4AB13B3F1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16980" xr2:uid="{336CA497-929E-8E43-ACC0-3AB4AB13B3F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -191,13 +191,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -211,7 +210,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,22 +585,22 @@
       <c r="G2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="J2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="N2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="11" t="s">
         <v>8</v>
       </c>
     </row>
@@ -610,161 +608,161 @@
       <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="5">
-        <v>4</v>
-      </c>
-      <c r="C3" s="6">
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3" s="5">
         <v>4</v>
       </c>
       <c r="E3" s="4">
         <v>1</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="6"/>
-      <c r="I3" s="13">
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="I3" s="12">
         <v>1</v>
       </c>
-      <c r="J3" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="K3" s="15"/>
-      <c r="M3" s="13">
+      <c r="J3" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="K3" s="14"/>
+      <c r="M3" s="12">
         <v>1</v>
       </c>
-      <c r="N3" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="O3" s="15"/>
+      <c r="N3" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="O3" s="14"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="5">
-        <v>4</v>
-      </c>
-      <c r="C4" s="6">
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5">
         <v>4</v>
       </c>
       <c r="E4" s="4">
         <v>2</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="6"/>
-      <c r="I4" s="13">
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="5"/>
+      <c r="I4" s="12">
         <v>2</v>
       </c>
-      <c r="J4" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="15"/>
-      <c r="M4" s="13">
+      <c r="J4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="14"/>
+      <c r="M4" s="12">
         <v>2</v>
       </c>
-      <c r="N4" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="O4" s="15"/>
+      <c r="N4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="O4" s="14"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="5">
-        <v>4</v>
-      </c>
-      <c r="C5" s="6">
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5">
         <v>4</v>
       </c>
       <c r="E5" s="4">
         <v>3</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="I5" s="13">
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="5"/>
+      <c r="I5" s="12">
         <v>3</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="K5" s="15"/>
-      <c r="M5" s="13">
+      <c r="J5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5" s="14"/>
+      <c r="M5" s="12">
         <v>3</v>
       </c>
-      <c r="N5" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="O5" s="15"/>
+      <c r="N5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="O5" s="14"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="19">
-        <v>4</v>
-      </c>
-      <c r="C6" s="6">
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5">
         <v>4</v>
       </c>
       <c r="E6" s="4">
         <v>4</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="6"/>
-      <c r="I6" s="13">
-        <v>4</v>
-      </c>
-      <c r="J6" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="K6" s="15"/>
-      <c r="M6" s="13">
-        <v>4</v>
-      </c>
-      <c r="N6" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="O6" s="15"/>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="I6" s="12">
+        <v>4</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="14"/>
+      <c r="M6" s="12">
+        <v>4</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="O6" s="14"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="8">
-        <v>4</v>
-      </c>
-      <c r="C7" s="9">
-        <v>4</v>
-      </c>
-      <c r="E7" s="7">
+      <c r="B7" s="7">
+        <v>4</v>
+      </c>
+      <c r="C7" s="8">
+        <v>4</v>
+      </c>
+      <c r="E7" s="6">
         <v>5</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="9"/>
-      <c r="I7" s="16">
+      <c r="F7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="8"/>
+      <c r="I7" s="15">
         <v>5</v>
       </c>
-      <c r="J7" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="K7" s="18"/>
-      <c r="M7" s="16">
+      <c r="J7" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="K7" s="17"/>
+      <c r="M7" s="15">
         <v>5</v>
       </c>
-      <c r="N7" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="O7" s="18"/>
+      <c r="N7" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="O7" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>